<commit_message>
feat: Phase 3+4 — voice input, unified AI entry, architecture cleanup
Phase 3.2: Voice integration in AIChatScreen
- Added mic button (replaces non-functional + button)
- isRecording state + handleVoiceInput toggle
- SpeechRecognitionService pipes ASR result to input

Phase 3.3: SmartBI + AI chat unified entry
- SmartBIStackNavigator NLQuery route → AIChatScreen
- AIChatScreen accepts both initialQuery and initialMessage params

Phase 4: Architecture cleanup
- Deleted GenerateHandlerConfigTool.java (338 lines dead code)
- Cleaned 5 stale Handler references in comments

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/python/smartbi/tests/test_complex_5sheets.xlsx
+++ b/backend/python/smartbi/tests/test_complex_5sheets.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2025年利润表" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="销售明细" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="部门预算对比" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="产品成本分析" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="待补充数据" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="2025年利润表" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="销售明细" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="部门预算对比" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="产品成本分析" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="待补充数据" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1021,31 +1021,31 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>宁波大润发</t>
+          <t>杭州联华</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>麻辣烫底料</t>
+          <t>火锅底料</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1kg/袋</t>
+          <t>250g/盒</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>673</v>
+        <v>217</v>
       </c>
       <c r="G4" t="n">
-        <v>19.23</v>
+        <v>43.87</v>
       </c>
       <c r="H4" t="n">
-        <v>12941.79</v>
+        <v>9519.790000000001</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>李四</t>
+          <t>张三</t>
         </is>
       </c>
     </row>
@@ -1060,31 +1060,31 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>杭州联华</t>
+          <t>宁波大润发</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>番茄底料</t>
+          <t>菌菇底料</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>500g/盒</t>
+          <t>500g/袋</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>491</v>
+        <v>703</v>
       </c>
       <c r="G5" t="n">
-        <v>30.9</v>
+        <v>26.72</v>
       </c>
       <c r="H5" t="n">
-        <v>15171.9</v>
+        <v>18784.16</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>李四</t>
+          <t>赵六</t>
         </is>
       </c>
     </row>
@@ -1099,7 +1099,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>温州永辉</t>
+          <t>杭州联华</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1109,21 +1109,21 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>250g/盒</t>
+          <t>500g/盒</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>117</v>
+        <v>931</v>
       </c>
       <c r="G6" t="n">
-        <v>37.12</v>
+        <v>29.29</v>
       </c>
       <c r="H6" t="n">
-        <v>4343.04</v>
+        <v>27268.99</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>李四</t>
+          <t>王五</t>
         </is>
       </c>
     </row>
@@ -1138,31 +1138,31 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>杭州联华</t>
+          <t>上海沃尔玛</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>番茄底料</t>
+          <t>酸菜鱼底料</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>250g/盒</t>
+          <t>500g/盒</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>907</v>
+        <v>793</v>
       </c>
       <c r="G7" t="n">
-        <v>15.91</v>
+        <v>22.3</v>
       </c>
       <c r="H7" t="n">
-        <v>14430.37</v>
+        <v>17683.9</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>李四</t>
+          <t>张三</t>
         </is>
       </c>
     </row>
@@ -1177,27 +1177,27 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>宁波大润发</t>
+          <t>温州永辉</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>麻辣烫底料</t>
+          <t>酸菜鱼底料</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>500g/袋</t>
+          <t>250g/盒</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>576</v>
+        <v>911</v>
       </c>
       <c r="G8" t="n">
-        <v>16.41</v>
+        <v>36.34</v>
       </c>
       <c r="H8" t="n">
-        <v>9452.16</v>
+        <v>33105.74</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
@@ -1216,12 +1216,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>宁波大润发</t>
+          <t>上海沃尔玛</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>火锅底料</t>
+          <t>麻辣烫底料</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -1230,13 +1230,13 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>158</v>
+        <v>226</v>
       </c>
       <c r="G9" t="n">
-        <v>27.9</v>
+        <v>18.2</v>
       </c>
       <c r="H9" t="n">
-        <v>4408.2</v>
+        <v>4113.2</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
@@ -1255,12 +1255,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>嘉兴世纪联华</t>
+          <t>宁波大润发</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>麻辣烫底料</t>
+          <t>火锅底料</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1269,13 +1269,13 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>364</v>
+        <v>950</v>
       </c>
       <c r="G10" t="n">
-        <v>33.94</v>
+        <v>38.34</v>
       </c>
       <c r="H10" t="n">
-        <v>12354.16</v>
+        <v>36423</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -1294,7 +1294,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>宁波大润发</t>
+          <t>杭州联华</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1308,13 +1308,13 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>893</v>
+        <v>856</v>
       </c>
       <c r="G11" t="n">
-        <v>37.87</v>
+        <v>16.31</v>
       </c>
       <c r="H11" t="n">
-        <v>33817.91</v>
+        <v>13961.36</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
@@ -1338,26 +1338,26 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>番茄底料</t>
+          <t>酸菜鱼底料</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>500g/盒</t>
+          <t>250g/盒</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>753</v>
+        <v>196</v>
       </c>
       <c r="G12" t="n">
-        <v>36.65</v>
+        <v>21.96</v>
       </c>
       <c r="H12" t="n">
-        <v>27597.45</v>
+        <v>4304.16</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>赵六</t>
+          <t>张三</t>
         </is>
       </c>
     </row>
@@ -1372,12 +1372,12 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>温州永辉</t>
+          <t>宁波大润发</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>菌菇底料</t>
+          <t>酸菜鱼底料</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1386,17 +1386,17 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>200</v>
+        <v>562</v>
       </c>
       <c r="G13" t="n">
-        <v>18.32</v>
+        <v>21.19</v>
       </c>
       <c r="H13" t="n">
-        <v>3664</v>
+        <v>11908.78</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>赵六</t>
+          <t>王五</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1416,31 +1416,31 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>上海沃尔玛</t>
+          <t>杭州联华</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>菌菇底料</t>
+          <t>麻辣烫底料</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>250g/盒</t>
+          <t>500g/袋</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>275</v>
+        <v>697</v>
       </c>
       <c r="G14" t="n">
-        <v>36.47</v>
+        <v>22.96</v>
       </c>
       <c r="H14" t="n">
-        <v>10029.25</v>
+        <v>16003.12</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>李四</t>
+          <t>张三</t>
         </is>
       </c>
     </row>
@@ -1460,26 +1460,26 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>麻辣烫底料</t>
+          <t>酸菜鱼底料</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1kg/袋</t>
+          <t>250g/盒</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>357</v>
+        <v>812</v>
       </c>
       <c r="G15" t="n">
-        <v>40.64</v>
+        <v>18.46</v>
       </c>
       <c r="H15" t="n">
-        <v>14508.48</v>
+        <v>14989.52</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>王五</t>
+          <t>李四</t>
         </is>
       </c>
     </row>
@@ -1494,31 +1494,31 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>嘉兴世纪联华</t>
+          <t>上海沃尔玛</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>菌菇底料</t>
+          <t>火锅底料</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1kg/袋</t>
+          <t>250g/盒</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>777</v>
+        <v>724</v>
       </c>
       <c r="G16" t="n">
-        <v>34.87</v>
+        <v>15.43</v>
       </c>
       <c r="H16" t="n">
-        <v>27093.99</v>
+        <v>11171.32</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>李四</t>
+          <t>王五</t>
         </is>
       </c>
     </row>
@@ -1538,26 +1538,26 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>麻辣烫底料</t>
+          <t>酸菜鱼底料</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1kg/袋</t>
+          <t>500g/袋</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>813</v>
+        <v>100</v>
       </c>
       <c r="G17" t="n">
-        <v>35.76</v>
+        <v>40.19</v>
       </c>
       <c r="H17" t="n">
-        <v>29072.88</v>
+        <v>4019</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>张三</t>
+          <t>王五</t>
         </is>
       </c>
     </row>
@@ -1572,27 +1572,27 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>杭州联华</t>
+          <t>上海沃尔玛</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>酸菜鱼底料</t>
+          <t>火锅底料</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>500g/袋</t>
+          <t>500g/盒</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>947</v>
+        <v>901</v>
       </c>
       <c r="G18" t="n">
-        <v>33.88</v>
+        <v>18.26</v>
       </c>
       <c r="H18" t="n">
-        <v>32084.36</v>
+        <v>16452.26</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
@@ -1611,31 +1611,31 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>嘉兴世纪联华</t>
+          <t>上海沃尔玛</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>火锅底料</t>
+          <t>番茄底料</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1kg/袋</t>
+          <t>500g/盒</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>242</v>
+        <v>829</v>
       </c>
       <c r="G19" t="n">
-        <v>26.1</v>
+        <v>18.6</v>
       </c>
       <c r="H19" t="n">
-        <v>6316.2</v>
+        <v>15419.4</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>王五</t>
+          <t>李四</t>
         </is>
       </c>
     </row>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>嘉兴世纪联华</t>
+          <t>杭州联华</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>番茄底料</t>
+          <t>酸菜鱼底料</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1664,17 +1664,17 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>756</v>
+        <v>988</v>
       </c>
       <c r="G20" t="n">
-        <v>24.11</v>
+        <v>30.43</v>
       </c>
       <c r="H20" t="n">
-        <v>18227.16</v>
+        <v>30064.84</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>李四</t>
+          <t>赵六</t>
         </is>
       </c>
     </row>
@@ -1689,7 +1689,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>杭州联华</t>
+          <t>上海沃尔玛</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1699,17 +1699,17 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>500g/盒</t>
+          <t>1kg/袋</t>
         </is>
       </c>
       <c r="F21" t="n">
-        <v>469</v>
+        <v>848</v>
       </c>
       <c r="G21" t="n">
-        <v>21.64</v>
+        <v>24.55</v>
       </c>
       <c r="H21" t="n">
-        <v>10149.16</v>
+        <v>20818.4</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
@@ -1728,12 +1728,12 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>上海沃尔玛</t>
+          <t>宁波大润发</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>菌菇底料</t>
+          <t>酸菜鱼底料</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1742,17 +1742,17 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>293</v>
+        <v>989</v>
       </c>
       <c r="G22" t="n">
-        <v>23.58</v>
+        <v>25.52</v>
       </c>
       <c r="H22" t="n">
-        <v>6908.94</v>
+        <v>25239.28</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>张三</t>
+          <t>赵六</t>
         </is>
       </c>
     </row>
@@ -1772,7 +1772,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>番茄底料</t>
+          <t>菌菇底料</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1781,17 +1781,17 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>975</v>
+        <v>290</v>
       </c>
       <c r="G23" t="n">
-        <v>38.46</v>
+        <v>15.36</v>
       </c>
       <c r="H23" t="n">
-        <v>37498.5</v>
+        <v>4454.4</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>张三</t>
+          <t>王五</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -1811,12 +1811,12 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>上海沃尔玛</t>
+          <t>嘉兴世纪联华</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>火锅底料</t>
+          <t>菌菇底料</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1825,17 +1825,17 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>117</v>
+        <v>661</v>
       </c>
       <c r="G24" t="n">
-        <v>27.59</v>
+        <v>43.22</v>
       </c>
       <c r="H24" t="n">
-        <v>3228.03</v>
+        <v>28568.42</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>张三</t>
+          <t>赵六</t>
         </is>
       </c>
     </row>
@@ -1850,31 +1850,31 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>上海沃尔玛</t>
+          <t>宁波大润发</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>番茄底料</t>
+          <t>酸菜鱼底料</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>500g/袋</t>
+          <t>1kg/袋</t>
         </is>
       </c>
       <c r="F25" t="n">
-        <v>671</v>
+        <v>742</v>
       </c>
       <c r="G25" t="n">
-        <v>18.93</v>
+        <v>29.89</v>
       </c>
       <c r="H25" t="n">
-        <v>12702.03</v>
+        <v>22178.38</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>王五</t>
+          <t>张三</t>
         </is>
       </c>
     </row>
@@ -1889,27 +1889,27 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>上海沃尔玛</t>
+          <t>杭州联华</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>火锅底料</t>
+          <t>麻辣烫底料</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>250g/盒</t>
+          <t>500g/袋</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>476</v>
+        <v>208</v>
       </c>
       <c r="G26" t="n">
-        <v>31.77</v>
+        <v>22.77</v>
       </c>
       <c r="H26" t="n">
-        <v>15122.52</v>
+        <v>4736.16</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
@@ -1928,27 +1928,27 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>宁波大润发</t>
+          <t>嘉兴世纪联华</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>番茄底料</t>
+          <t>菌菇底料</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>500g/盒</t>
+          <t>500g/袋</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>878</v>
+        <v>148</v>
       </c>
       <c r="G27" t="n">
-        <v>37.91</v>
+        <v>36.14</v>
       </c>
       <c r="H27" t="n">
-        <v>33284.98</v>
+        <v>5348.72</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
@@ -1972,22 +1972,22 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>酸菜鱼底料</t>
+          <t>番茄底料</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>500g/盒</t>
+          <t>500g/袋</t>
         </is>
       </c>
       <c r="F28" t="n">
-        <v>406</v>
+        <v>149</v>
       </c>
       <c r="G28" t="n">
-        <v>25.87</v>
+        <v>23.08</v>
       </c>
       <c r="H28" t="n">
-        <v>10503.22</v>
+        <v>3438.92</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
@@ -2006,31 +2006,31 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>宁波大润发</t>
+          <t>温州永辉</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>火锅底料</t>
+          <t>菌菇底料</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>1kg/袋</t>
+          <t>250g/盒</t>
         </is>
       </c>
       <c r="F29" t="n">
-        <v>340</v>
+        <v>560</v>
       </c>
       <c r="G29" t="n">
-        <v>31.08</v>
+        <v>35.27</v>
       </c>
       <c r="H29" t="n">
-        <v>10567.2</v>
+        <v>19751.2</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>赵六</t>
+          <t>王五</t>
         </is>
       </c>
     </row>
@@ -2045,7 +2045,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>上海沃尔玛</t>
+          <t>嘉兴世纪联华</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -2059,17 +2059,17 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>979</v>
+        <v>474</v>
       </c>
       <c r="G30" t="n">
-        <v>30.67</v>
+        <v>28.26</v>
       </c>
       <c r="H30" t="n">
-        <v>30025.93</v>
+        <v>13395.24</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>张三</t>
+          <t>王五</t>
         </is>
       </c>
     </row>
@@ -2084,27 +2084,27 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>嘉兴世纪联华</t>
+          <t>上海沃尔玛</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>菌菇底料</t>
+          <t>麻辣烫底料</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>250g/盒</t>
+          <t>500g/袋</t>
         </is>
       </c>
       <c r="F31" t="n">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="G31" t="n">
-        <v>35.46</v>
+        <v>16.11</v>
       </c>
       <c r="H31" t="n">
-        <v>8404.02</v>
+        <v>3834.18</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
@@ -2123,7 +2123,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>嘉兴世纪联华</t>
+          <t>杭州联华</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -2133,17 +2133,17 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>1kg/袋</t>
+          <t>500g/盒</t>
         </is>
       </c>
       <c r="F32" t="n">
-        <v>289</v>
+        <v>712</v>
       </c>
       <c r="G32" t="n">
-        <v>26.43</v>
+        <v>44.4</v>
       </c>
       <c r="H32" t="n">
-        <v>7638.27</v>
+        <v>31612.8</v>
       </c>
       <c r="I32" t="inlineStr">
         <is>
@@ -2162,27 +2162,27 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>杭州联华</t>
+          <t>宁波大润发</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>酸菜鱼底料</t>
+          <t>番茄底料</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>500g/盒</t>
+          <t>1kg/袋</t>
         </is>
       </c>
       <c r="F33" t="n">
-        <v>364</v>
+        <v>509</v>
       </c>
       <c r="G33" t="n">
-        <v>43.92</v>
+        <v>40.33</v>
       </c>
       <c r="H33" t="n">
-        <v>15986.88</v>
+        <v>20527.97</v>
       </c>
       <c r="I33" t="inlineStr">
         <is>
@@ -2211,26 +2211,26 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>麻辣烫底料</t>
+          <t>火锅底料</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>500g/盒</t>
+          <t>250g/盒</t>
         </is>
       </c>
       <c r="F34" t="n">
-        <v>971</v>
+        <v>216</v>
       </c>
       <c r="G34" t="n">
-        <v>32.68</v>
+        <v>18</v>
       </c>
       <c r="H34" t="n">
-        <v>31732.28</v>
+        <v>3888</v>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>赵六</t>
+          <t>张三</t>
         </is>
       </c>
     </row>
@@ -2245,31 +2245,31 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>温州永辉</t>
+          <t>上海沃尔玛</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>火锅底料</t>
+          <t>菌菇底料</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>250g/盒</t>
+          <t>500g/盒</t>
         </is>
       </c>
       <c r="F35" t="n">
-        <v>549</v>
+        <v>825</v>
       </c>
       <c r="G35" t="n">
-        <v>33.51</v>
+        <v>25.85</v>
       </c>
       <c r="H35" t="n">
-        <v>18396.99</v>
+        <v>21326.25</v>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>李四</t>
+          <t>赵六</t>
         </is>
       </c>
     </row>
@@ -2289,7 +2289,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>酸菜鱼底料</t>
+          <t>麻辣烫底料</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -2298,17 +2298,17 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>777</v>
+        <v>715</v>
       </c>
       <c r="G36" t="n">
-        <v>33.66</v>
+        <v>26.99</v>
       </c>
       <c r="H36" t="n">
-        <v>26153.82</v>
+        <v>19297.85</v>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>李四</t>
+          <t>赵六</t>
         </is>
       </c>
     </row>
@@ -2328,22 +2328,22 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>酸菜鱼底料</t>
+          <t>番茄底料</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>1kg/袋</t>
+          <t>250g/盒</t>
         </is>
       </c>
       <c r="F37" t="n">
-        <v>617</v>
+        <v>455</v>
       </c>
       <c r="G37" t="n">
-        <v>37.83</v>
+        <v>17.34</v>
       </c>
       <c r="H37" t="n">
-        <v>23341.11</v>
+        <v>7889.7</v>
       </c>
       <c r="I37" t="inlineStr">
         <is>
@@ -2362,27 +2362,27 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>宁波大润发</t>
+          <t>上海沃尔玛</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>菌菇底料</t>
+          <t>火锅底料</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>500g/盒</t>
+          <t>250g/盒</t>
         </is>
       </c>
       <c r="F38" t="n">
-        <v>505</v>
+        <v>328</v>
       </c>
       <c r="G38" t="n">
-        <v>34.62</v>
+        <v>25.98</v>
       </c>
       <c r="H38" t="n">
-        <v>17483.1</v>
+        <v>8521.440000000001</v>
       </c>
       <c r="I38" t="inlineStr">
         <is>
@@ -2415,17 +2415,17 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>823</v>
+        <v>875</v>
       </c>
       <c r="G39" t="n">
-        <v>33.37</v>
+        <v>15.93</v>
       </c>
       <c r="H39" t="n">
-        <v>27463.51</v>
+        <v>13938.75</v>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>李四</t>
+          <t>赵六</t>
         </is>
       </c>
     </row>
@@ -2450,17 +2450,17 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>1kg/袋</t>
+          <t>250g/盒</t>
         </is>
       </c>
       <c r="F40" t="n">
-        <v>516</v>
+        <v>340</v>
       </c>
       <c r="G40" t="n">
-        <v>27.11</v>
+        <v>19.88</v>
       </c>
       <c r="H40" t="n">
-        <v>13988.76</v>
+        <v>6759.2</v>
       </c>
       <c r="I40" t="inlineStr">
         <is>
@@ -2484,22 +2484,22 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>酸菜鱼底料</t>
+          <t>麻辣烫底料</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>250g/盒</t>
+          <t>500g/袋</t>
         </is>
       </c>
       <c r="F41" t="n">
-        <v>254</v>
+        <v>782</v>
       </c>
       <c r="G41" t="n">
-        <v>44.92</v>
+        <v>35.62</v>
       </c>
       <c r="H41" t="n">
-        <v>11409.68</v>
+        <v>27854.84</v>
       </c>
       <c r="I41" t="inlineStr">
         <is>
@@ -2518,27 +2518,27 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>上海沃尔玛</t>
+          <t>宁波大润发</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>火锅底料</t>
+          <t>酸菜鱼底料</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>500g/袋</t>
+          <t>1kg/袋</t>
         </is>
       </c>
       <c r="F42" t="n">
-        <v>752</v>
+        <v>611</v>
       </c>
       <c r="G42" t="n">
-        <v>23.27</v>
+        <v>34.74</v>
       </c>
       <c r="H42" t="n">
-        <v>17499.04</v>
+        <v>21226.14</v>
       </c>
       <c r="I42" t="inlineStr">
         <is>
@@ -2557,31 +2557,31 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>嘉兴世纪联华</t>
+          <t>温州永辉</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>麻辣烫底料</t>
+          <t>火锅底料</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>250g/盒</t>
+          <t>500g/盒</t>
         </is>
       </c>
       <c r="F43" t="n">
-        <v>355</v>
+        <v>825</v>
       </c>
       <c r="G43" t="n">
-        <v>31.14</v>
+        <v>41.83</v>
       </c>
       <c r="H43" t="n">
-        <v>11054.7</v>
+        <v>34509.75</v>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>张三</t>
+          <t>李四</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
@@ -2601,27 +2601,27 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>宁波大润发</t>
+          <t>嘉兴世纪联华</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>菌菇底料</t>
+          <t>麻辣烫底料</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>1kg/袋</t>
+          <t>500g/袋</t>
         </is>
       </c>
       <c r="F44" t="n">
-        <v>546</v>
+        <v>568</v>
       </c>
       <c r="G44" t="n">
-        <v>35.04</v>
+        <v>15.12</v>
       </c>
       <c r="H44" t="n">
-        <v>19131.84</v>
+        <v>8588.16</v>
       </c>
       <c r="I44" t="inlineStr">
         <is>
@@ -2645,26 +2645,26 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>酸菜鱼底料</t>
+          <t>番茄底料</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>500g/盒</t>
+          <t>250g/盒</t>
         </is>
       </c>
       <c r="F45" t="n">
-        <v>681</v>
+        <v>596</v>
       </c>
       <c r="G45" t="n">
-        <v>30.08</v>
+        <v>16.4</v>
       </c>
       <c r="H45" t="n">
-        <v>20484.48</v>
+        <v>9774.4</v>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>张三</t>
+          <t>赵六</t>
         </is>
       </c>
     </row>
@@ -2679,31 +2679,31 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>杭州联华</t>
+          <t>宁波大润发</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>酸菜鱼底料</t>
+          <t>菌菇底料</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>500g/盒</t>
+          <t>1kg/袋</t>
         </is>
       </c>
       <c r="F46" t="n">
-        <v>293</v>
+        <v>142</v>
       </c>
       <c r="G46" t="n">
-        <v>28.8</v>
+        <v>36.82</v>
       </c>
       <c r="H46" t="n">
-        <v>8438.4</v>
+        <v>5228.44</v>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>赵六</t>
+          <t>王五</t>
         </is>
       </c>
     </row>
@@ -2718,31 +2718,31 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>上海沃尔玛</t>
+          <t>嘉兴世纪联华</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>番茄底料</t>
+          <t>火锅底料</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>1kg/袋</t>
+          <t>500g/盒</t>
         </is>
       </c>
       <c r="F47" t="n">
-        <v>516</v>
+        <v>173</v>
       </c>
       <c r="G47" t="n">
-        <v>41.9</v>
+        <v>23.97</v>
       </c>
       <c r="H47" t="n">
-        <v>21620.4</v>
+        <v>4146.81</v>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>李四</t>
+          <t>赵六</t>
         </is>
       </c>
     </row>
@@ -2757,31 +2757,31 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>嘉兴世纪联华</t>
+          <t>宁波大润发</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>火锅底料</t>
+          <t>麻辣烫底料</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>250g/盒</t>
+          <t>500g/盒</t>
         </is>
       </c>
       <c r="F48" t="n">
-        <v>895</v>
+        <v>870</v>
       </c>
       <c r="G48" t="n">
-        <v>44.36</v>
+        <v>37.04</v>
       </c>
       <c r="H48" t="n">
-        <v>39702.2</v>
+        <v>32224.8</v>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>李四</t>
+          <t>张三</t>
         </is>
       </c>
     </row>
@@ -2796,31 +2796,31 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>上海沃尔玛</t>
+          <t>温州永辉</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>酸菜鱼底料</t>
+          <t>番茄底料</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>500g/盒</t>
+          <t>500g/袋</t>
         </is>
       </c>
       <c r="F49" t="n">
-        <v>515</v>
+        <v>885</v>
       </c>
       <c r="G49" t="n">
-        <v>35.21</v>
+        <v>19.39</v>
       </c>
       <c r="H49" t="n">
-        <v>18133.15</v>
+        <v>17160.15</v>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>李四</t>
+          <t>王五</t>
         </is>
       </c>
     </row>
@@ -2835,31 +2835,31 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>嘉兴世纪联华</t>
+          <t>温州永辉</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>麻辣烫底料</t>
+          <t>火锅底料</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>500g/盒</t>
+          <t>1kg/袋</t>
         </is>
       </c>
       <c r="F50" t="n">
-        <v>502</v>
+        <v>335</v>
       </c>
       <c r="G50" t="n">
-        <v>19.39</v>
+        <v>28.79</v>
       </c>
       <c r="H50" t="n">
-        <v>9733.780000000001</v>
+        <v>9644.65</v>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>赵六</t>
+          <t>张三</t>
         </is>
       </c>
     </row>
@@ -2874,27 +2874,27 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>上海沃尔玛</t>
+          <t>宁波大润发</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>酸菜鱼底料</t>
+          <t>番茄底料</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>500g/盒</t>
+          <t>500g/袋</t>
         </is>
       </c>
       <c r="F51" t="n">
-        <v>165</v>
+        <v>411</v>
       </c>
       <c r="G51" t="n">
-        <v>31.99</v>
+        <v>18.15</v>
       </c>
       <c r="H51" t="n">
-        <v>5278.35</v>
+        <v>7459.65</v>
       </c>
       <c r="I51" t="inlineStr">
         <is>
@@ -2913,31 +2913,31 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>温州永辉</t>
+          <t>宁波大润发</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>菌菇底料</t>
+          <t>酸菜鱼底料</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>1kg/袋</t>
+          <t>250g/盒</t>
         </is>
       </c>
       <c r="F52" t="n">
-        <v>739</v>
+        <v>212</v>
       </c>
       <c r="G52" t="n">
-        <v>40.98</v>
+        <v>22.42</v>
       </c>
       <c r="H52" t="n">
-        <v>30284.22</v>
+        <v>4753.04</v>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>赵六</t>
+          <t>李四</t>
         </is>
       </c>
     </row>
@@ -2952,31 +2952,31 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>宁波大润发</t>
+          <t>嘉兴世纪联华</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>酸菜鱼底料</t>
+          <t>菌菇底料</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>500g/盒</t>
+          <t>500g/袋</t>
         </is>
       </c>
       <c r="F53" t="n">
-        <v>397</v>
+        <v>968</v>
       </c>
       <c r="G53" t="n">
-        <v>21.81</v>
+        <v>27.01</v>
       </c>
       <c r="H53" t="n">
-        <v>8658.57</v>
+        <v>26145.68</v>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>李四</t>
+          <t>赵六</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">

</xml_diff>